<commit_message>
Feat: Make lookback window configurable and add Monthly execution mode
</commit_message>
<xml_diff>
--- a/input/products_to_track.xlsx
+++ b/input/products_to_track.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harsh.sharma2\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62309536-A140-49BF-8CD8-92A395A13417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-14565" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="106">
   <si>
     <t>NAV Code</t>
   </si>
@@ -151,9 +157,6 @@
     <t>Tesco Finest Air Dried Crumbed Ham 130g</t>
   </si>
   <si>
-    <t>Tesco FInest Dry Cured Finely Sliced Ham 130g</t>
-  </si>
-  <si>
     <t>Tesco Finest Dry Cured Old English Ham 130g</t>
   </si>
   <si>
@@ -172,158 +175,176 @@
     <t>Deli Ox Tongue 100g</t>
   </si>
   <si>
-    <t>https://www.tesco.com/shop/en-GB/products/276414756</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/316060787</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/311807538</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/315838817</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/315831427</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/312215577</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/303880749</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/303881218</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/315967474</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/276415346</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/315837790</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/299957350</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/303881247</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/315860980</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/299955783</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/303880703</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/316177140</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/316189379</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/316199148</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/315961780</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/316198881</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/305974463</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/315956936</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/316064247</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/316192340</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/310666982</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/314691737</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/299955685</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/303880473</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/299955800</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/299955823</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/316173639</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/320562605</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/314708576</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/321660977</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/321340550</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/321666320</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/323422525</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/317542720</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/317535887</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/317046904</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/317296383</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/316055745</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/317197788</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/317196432</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/320542917</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/322158298</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/312712723</t>
-  </si>
-  <si>
-    <t>https://www.tesco.com/shop/en-GB/products/312208094</t>
+    <t>Tesco British Crumbed Ham Slices 400g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Crumbed Ham Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Roast Beef Slices 90g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Wafer Thin Roast Chicken Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Roast Chicken Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Prime Cuts Roast Chicken &amp; Stuffing 4 Slices 100G - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Honey Roast Ham Slices 400g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Wafer Thin Honey Roast Ham Slices 125g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Prime Cuts Honey Roast Ham 6 Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Honey Roast Ham Slices 400g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Wafer Thin Honey Roast Ham Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Pastrami Slices 100g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Wafer Thin Smoked Ham Slices 125g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Pork &amp; Egg Roll Slices 125g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Eastmans Cooked Ham Slices 125g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Eastmans Wafer Thin Cooked Chicken Slices 125g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Cooked Ham Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Garlic Sausage Slices 125g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Smoked Ham 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Wafer Thin Smoked Ham Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Wafer Thin Cooked Ham Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Eastmans Corned Beef Slices 150g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Thick Cut Honey &amp; Mustard Ham Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Lean Ham on the Bone Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Peppered Ham Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Cumberland Sausage Slices 150g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Premier Deli Roast Turkey Breast Slices 125g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Eastmans Cooked Ham Slices 400g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Eastmans Wafer Thin Cooked Ham Slices 400g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Eastmans Pork Luncheon Meat Slices 250g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Eastmans Cooked Chicken Roll Slices 250g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Pork Lunch Tongue Slices 120g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Roast Pork Loin Slices 100g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco British Corned Beef 110g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Wafer Thin Cooked Ham 125g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Cooked Ham 400g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Wafer Thin Cooked Ham 400g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Core British Roast Chicken and Stuffing 100g</t>
+  </si>
+  <si>
+    <t>Tesco Finest Dry-Cured Ham on the Bone Slices 200g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Finest Dry Cured Cooked Ham Slices 130g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Finest Dry Cured Honey Roast Ham Slices 130g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Finest Dry Cured Oak Smoked Ham Slices 130g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Finest Dry Cured Crumbed Ham Slices 130g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Finest Dry Cured 'Old English Ham' Slices 130g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Finest Slow Cooked Roast Beef Topside Slices 90g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Finest Dry Cured Ham on the Bone Slices 130g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Finest Deli Herb Crusted Ham Slices 130g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Deli Roast Turkey Breast 120G - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Deli Ox Tongue 100G - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Deli Corned Beef 140g</t>
+  </si>
+  <si>
+    <t>Tesco Corned Beef 4 Slices 140g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Tesco Finest Hickory Smoked Brisket 70g</t>
+  </si>
+  <si>
+    <t>Tesco Finest Hickory Smoked Brisket 70g - Tesco Groceries</t>
+  </si>
+  <si>
+    <t>Core EU Cooked Beef 125g</t>
+  </si>
+  <si>
+    <t>Tesco Cooked Beef Slices 125g - Tesco Groceries</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -373,13 +394,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -417,7 +446,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -451,6 +480,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -485,9 +515,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -660,11 +691,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C54"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.88671875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -675,7 +711,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>10011247</v>
       </c>
@@ -683,10 +719,10 @@
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>10100822</v>
       </c>
@@ -694,10 +730,10 @@
         <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>10100556</v>
       </c>
@@ -705,10 +741,10 @@
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>10100820</v>
       </c>
@@ -716,10 +752,10 @@
         <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>10100819</v>
       </c>
@@ -727,10 +763,10 @@
         <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>10026259</v>
       </c>
@@ -738,10 +774,10 @@
         <v>8</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>10020977</v>
       </c>
@@ -749,10 +785,10 @@
         <v>9</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>10020975</v>
       </c>
@@ -760,10 +796,10 @@
         <v>10</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10100823</v>
       </c>
@@ -771,10 +807,10 @@
         <v>11</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10021822</v>
       </c>
@@ -782,10 +818,10 @@
         <v>12</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10100826</v>
       </c>
@@ -793,10 +829,10 @@
         <v>13</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>10018205</v>
       </c>
@@ -804,10 +840,10 @@
         <v>14</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>10020973</v>
       </c>
@@ -815,10 +851,10 @@
         <v>15</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>10106830</v>
       </c>
@@ -826,10 +862,10 @@
         <v>16</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>10025360</v>
       </c>
@@ -837,10 +873,10 @@
         <v>17</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>10020950</v>
       </c>
@@ -848,10 +884,10 @@
         <v>18</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>10100825</v>
       </c>
@@ -859,10 +895,10 @@
         <v>19</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>10100736</v>
       </c>
@@ -870,10 +906,10 @@
         <v>20</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>10100824</v>
       </c>
@@ -881,10 +917,10 @@
         <v>21</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>10100827</v>
       </c>
@@ -892,10 +928,10 @@
         <v>22</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>10100828</v>
       </c>
@@ -903,10 +939,10 @@
         <v>23</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>10023670</v>
       </c>
@@ -914,10 +950,10 @@
         <v>24</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>10106831</v>
       </c>
@@ -925,10 +961,10 @@
         <v>25</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>10100829</v>
       </c>
@@ -936,10 +972,10 @@
         <v>26</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>10100831</v>
       </c>
@@ -947,10 +983,10 @@
         <v>27</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>10100717</v>
       </c>
@@ -958,10 +994,10 @@
         <v>28</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>10100358</v>
       </c>
@@ -969,10 +1005,10 @@
         <v>29</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>10025359</v>
       </c>
@@ -980,10 +1016,10 @@
         <v>30</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>10020949</v>
       </c>
@@ -991,10 +1027,10 @@
         <v>31</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>10018180</v>
       </c>
@@ -1002,10 +1038,10 @@
         <v>32</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>10018181</v>
       </c>
@@ -1013,10 +1049,10 @@
         <v>33</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>10100821</v>
       </c>
@@ -1024,10 +1060,10 @@
         <v>34</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>10101213</v>
       </c>
@@ -1035,10 +1071,10 @@
         <v>35</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>10101339</v>
       </c>
@@ -1046,10 +1082,10 @@
         <v>36</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>10101397</v>
       </c>
@@ -1057,10 +1093,10 @@
         <v>37</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>10101398</v>
       </c>
@@ -1068,10 +1104,10 @@
         <v>38</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>10101399</v>
       </c>
@@ -1079,192 +1115,231 @@
         <v>39</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>10026259</v>
+      </c>
+      <c r="B39" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39">
+      <c r="C39" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40">
         <v>10105591</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>40</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
-      <c r="A40">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41">
         <v>10101060</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>41</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C41" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
-      <c r="A41">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42">
         <v>10101061</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>42</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C42" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
-      <c r="A42">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43">
         <v>10101309</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>43</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C43" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
-      <c r="A43">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44">
         <v>10101063</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B44" t="s">
         <v>44</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C44" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
-      <c r="A44">
-        <v>10101241</v>
-      </c>
-      <c r="B44" t="s">
-        <v>45</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>10101310</v>
       </c>
       <c r="B45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>10101311</v>
       </c>
       <c r="B46" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>10101216</v>
       </c>
       <c r="B47" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>10102784</v>
       </c>
       <c r="B48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>10100121</v>
       </c>
       <c r="B49" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>10100122</v>
       </c>
       <c r="B50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C50" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>10102782</v>
+      </c>
+      <c r="B51" t="s">
         <v>100</v>
       </c>
+      <c r="C51" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>10101446</v>
+      </c>
+      <c r="B52" t="s">
+        <v>102</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>10100735</v>
+      </c>
+      <c r="B53" t="s">
+        <v>104</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C54" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1"/>
-    <hyperlink ref="C3" r:id="rId2"/>
-    <hyperlink ref="C4" r:id="rId3"/>
-    <hyperlink ref="C5" r:id="rId4"/>
-    <hyperlink ref="C6" r:id="rId5"/>
-    <hyperlink ref="C7" r:id="rId6"/>
-    <hyperlink ref="C8" r:id="rId7"/>
-    <hyperlink ref="C9" r:id="rId8"/>
-    <hyperlink ref="C10" r:id="rId9"/>
-    <hyperlink ref="C11" r:id="rId10"/>
-    <hyperlink ref="C12" r:id="rId11"/>
-    <hyperlink ref="C13" r:id="rId12"/>
-    <hyperlink ref="C14" r:id="rId13"/>
-    <hyperlink ref="C15" r:id="rId14"/>
-    <hyperlink ref="C16" r:id="rId15"/>
-    <hyperlink ref="C17" r:id="rId16"/>
-    <hyperlink ref="C18" r:id="rId17"/>
-    <hyperlink ref="C19" r:id="rId18"/>
-    <hyperlink ref="C20" r:id="rId19"/>
-    <hyperlink ref="C21" r:id="rId20"/>
-    <hyperlink ref="C22" r:id="rId21"/>
-    <hyperlink ref="C23" r:id="rId22"/>
-    <hyperlink ref="C24" r:id="rId23"/>
-    <hyperlink ref="C25" r:id="rId24"/>
-    <hyperlink ref="C26" r:id="rId25"/>
-    <hyperlink ref="C27" r:id="rId26"/>
-    <hyperlink ref="C28" r:id="rId27"/>
-    <hyperlink ref="C29" r:id="rId28"/>
-    <hyperlink ref="C30" r:id="rId29"/>
-    <hyperlink ref="C31" r:id="rId30"/>
-    <hyperlink ref="C32" r:id="rId31"/>
-    <hyperlink ref="C33" r:id="rId32"/>
-    <hyperlink ref="C34" r:id="rId33"/>
-    <hyperlink ref="C35" r:id="rId34"/>
-    <hyperlink ref="C36" r:id="rId35"/>
-    <hyperlink ref="C37" r:id="rId36"/>
-    <hyperlink ref="C38" r:id="rId37"/>
-    <hyperlink ref="C39" r:id="rId38"/>
-    <hyperlink ref="C40" r:id="rId39"/>
-    <hyperlink ref="C41" r:id="rId40"/>
-    <hyperlink ref="C42" r:id="rId41"/>
-    <hyperlink ref="C43" r:id="rId42"/>
-    <hyperlink ref="C44" r:id="rId43"/>
-    <hyperlink ref="C45" r:id="rId44"/>
-    <hyperlink ref="C46" r:id="rId45"/>
-    <hyperlink ref="C47" r:id="rId46"/>
-    <hyperlink ref="C48" r:id="rId47"/>
-    <hyperlink ref="C49" r:id="rId48"/>
-    <hyperlink ref="C50" r:id="rId49"/>
+    <hyperlink ref="C2" r:id="rId1" display="https://www.tesco.com/shop/en-GB/products/276414756" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C3" r:id="rId2" display="https://www.tesco.com/shop/en-GB/products/316060787" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="C4" r:id="rId3" display="https://www.tesco.com/shop/en-GB/products/311807538" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="C5" r:id="rId4" display="https://www.tesco.com/shop/en-GB/products/315838817" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="C6" r:id="rId5" display="https://www.tesco.com/shop/en-GB/products/315831427" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="C7" r:id="rId6" display="https://www.tesco.com/shop/en-GB/products/312215577" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="C8" r:id="rId7" display="https://www.tesco.com/shop/en-GB/products/303880749" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="C9" r:id="rId8" display="https://www.tesco.com/shop/en-GB/products/303881218" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="C10" r:id="rId9" display="https://www.tesco.com/shop/en-GB/products/315967474" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="C11" r:id="rId10" display="https://www.tesco.com/shop/en-GB/products/276415346" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="C12" r:id="rId11" display="https://www.tesco.com/shop/en-GB/products/315837790" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="C13" r:id="rId12" display="https://www.tesco.com/shop/en-GB/products/299957350" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="C14" r:id="rId13" display="https://www.tesco.com/shop/en-GB/products/303881247" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="C15" r:id="rId14" display="https://www.tesco.com/shop/en-GB/products/315860980" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="C16" r:id="rId15" display="https://www.tesco.com/shop/en-GB/products/299955783" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="C17" r:id="rId16" display="https://www.tesco.com/shop/en-GB/products/303880703" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="C18" r:id="rId17" display="https://www.tesco.com/shop/en-GB/products/316177140" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="C19" r:id="rId18" display="https://www.tesco.com/shop/en-GB/products/316189379" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="C20" r:id="rId19" display="https://www.tesco.com/shop/en-GB/products/316199148" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="C21" r:id="rId20" display="https://www.tesco.com/shop/en-GB/products/315961780" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="C22" r:id="rId21" display="https://www.tesco.com/shop/en-GB/products/316198881" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="C23" r:id="rId22" display="https://www.tesco.com/shop/en-GB/products/305974463" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="C24" r:id="rId23" display="https://www.tesco.com/shop/en-GB/products/315956936" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="C25" r:id="rId24" display="https://www.tesco.com/shop/en-GB/products/316064247" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="C26" r:id="rId25" display="https://www.tesco.com/shop/en-GB/products/316192340" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="C27" r:id="rId26" display="https://www.tesco.com/shop/en-GB/products/310666982" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="C28" r:id="rId27" display="https://www.tesco.com/shop/en-GB/products/314691737" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="C29" r:id="rId28" display="https://www.tesco.com/shop/en-GB/products/299955685" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="C30" r:id="rId29" display="https://www.tesco.com/shop/en-GB/products/303880473" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="C31" r:id="rId30" display="https://www.tesco.com/shop/en-GB/products/299955800" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="C32" r:id="rId31" display="https://www.tesco.com/shop/en-GB/products/299955823" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="C33" r:id="rId32" display="https://www.tesco.com/shop/en-GB/products/316173639" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="C34" r:id="rId33" display="https://www.tesco.com/shop/en-GB/products/320562605" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="C35" r:id="rId34" display="https://www.tesco.com/shop/en-GB/products/314708576" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="C36" r:id="rId35" display="https://www.tesco.com/shop/en-GB/products/321660977" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="C37" r:id="rId36" display="https://www.tesco.com/shop/en-GB/products/321340550" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="C38" r:id="rId37" display="https://www.tesco.com/shop/en-GB/products/321666320" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="C39" r:id="rId38" display="https://www.tesco.com/shop/en-GB/products/323422525" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="C40" r:id="rId39" display="https://www.tesco.com/shop/en-GB/products/317542720" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="C41" r:id="rId40" display="https://www.tesco.com/shop/en-GB/products/317535887" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="C42" r:id="rId41" display="https://www.tesco.com/shop/en-GB/products/317046904" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="C43" r:id="rId42" display="https://www.tesco.com/shop/en-GB/products/317296383" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="C44" r:id="rId43" display="https://www.tesco.com/shop/en-GB/products/316055745" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="C45" r:id="rId44" display="https://www.tesco.com/shop/en-GB/products/317197788" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="C46" r:id="rId45" display="https://www.tesco.com/shop/en-GB/products/317196432" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="C47" r:id="rId46" display="https://www.tesco.com/shop/en-GB/products/320542917" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="C48" r:id="rId47" display="https://www.tesco.com/shop/en-GB/products/322158298" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="C49" r:id="rId48" display="https://www.tesco.com/shop/en-GB/products/312712723" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="C50" r:id="rId49" display="https://www.tesco.com/shop/en-GB/products/312208094?_gl=1*v1t3q1*_up*MQ..*_ga*MTA5NzU5MjA1NC4xNzg3ODQxMDY5*_ga_H653QXESTP*czE3ODc4NDEwNjkkbzEkZzAkdDE3ODc4NDEwNjkkajYwJGwwJGgxMDk1NTMwMzA.*_ga_33B19D36CY*czE3ODc4NDEwNjkkbzEkZzEkdDE3ODc4NDQzNDkkajYwJGwwJGgyMDQ4NjM4OTgy" xr:uid="{7F934D27-9B79-4018-A8A5-13E31598FA66}"/>
+    <hyperlink ref="C51" r:id="rId50" display="https://www.tesco.com/shop/en-GB/products/322259207?_gl=1*1uohn03*_up*MQ..*_ga*MTEzNTk3ODg3LjE3ODgyNDcyNTg.*_ga_H653QXESTP*czE3ODgyNDcyNTckbzEkZzAkdDE3ODgyNDc2NDkkajYwJGwwJGgxMTY3NDc4NTg2*_ga_33B19D36CY*czE3ODgyNTAxODUkbzIkZzAkdDE3ODgyNTAxODUkajYwJGwwJGgxODg5NTUwMzEw" xr:uid="{1EBAC078-272B-4209-BE84-DDCD2D0997CF}"/>
+    <hyperlink ref="C52" r:id="rId51" display="https://www.tesco.com/shop/en-GB/products/321838699?msockid=398af264865b6a3d1f58e5ec87856b25" xr:uid="{117B3758-8F66-49FA-A000-5036FBEC7230}"/>
+    <hyperlink ref="C53" r:id="rId52" display="https://www.tesco.com/shop/en-GB/products/316067316?msockid=398af264865b6a3d1f58e5ec87856b25" xr:uid="{18BD8A3A-0117-4B5B-8FB2-43581E67C4CD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>